<commit_message>
merge code from main branch
</commit_message>
<xml_diff>
--- a/nightwatch/test-data-result.xlsx
+++ b/nightwatch/test-data-result.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:K26"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -433,151 +433,40 @@
       <c r="K1" t="str">
         <v>Trạng thái (Pass/Fail)</v>
       </c>
-      <c r="L1" t="str">
-        <v>__EMPTY</v>
-      </c>
-      <c r="M1" t="str">
-        <v>__EMPTY_1</v>
-      </c>
-      <c r="N1" t="str">
-        <v>__EMPTY_2</v>
-      </c>
-      <c r="O1" t="str">
-        <v>__EMPTY_3</v>
-      </c>
-      <c r="P1" t="str">
-        <v>__EMPTY_4</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>__EMPTY_5</v>
-      </c>
-      <c r="R1" t="str">
-        <v>__EMPTY_6</v>
-      </c>
-      <c r="S1" t="str">
-        <v>__EMPTY_7</v>
-      </c>
-      <c r="T1" t="str">
-        <v>__EMPTY_8</v>
-      </c>
-      <c r="U1" t="str">
-        <v>__EMPTY_9</v>
-      </c>
-      <c r="V1" t="str">
-        <v>__EMPTY_10</v>
-      </c>
-      <c r="W1" t="str">
-        <v>__EMPTY_11</v>
-      </c>
-      <c r="X1" t="str">
-        <v>__EMPTY_12</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>__EMPTY_13</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>__EMPTY_14</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>__EMPTY_15</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>__EMPTY_16</v>
-      </c>
-    </row>
-    <row r="2" xml:space="preserve">
+    </row>
+    <row r="2">
       <c r="A2" t="str">
-        <v>TC02</v>
+        <v>TC01</v>
       </c>
       <c r="B2" t="str">
-        <v>Kiểm tra hiển thị trang Liên hệ</v>
+        <v>Kiểm tra truy cập trang chủ</v>
       </c>
       <c r="C2" t="str">
-        <v>Đảm bảo trang Liên hệ có thông tin liên lạc</v>
+        <v>Xác nhận trang chủ có thể truy cập được và hiển thị đầy đủ</v>
       </c>
       <c r="D2" t="str">
-        <v>Click menu/mục tương ứng</v>
-      </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Mở trình duyệt_x000d_
-2. Truy cập trang https://actvn.edu.vn_x000d_
-3. Hover vào mục 'Giới thiệu' trên navbar_x000d_
-4. Click vào mục 'Liên hệ'</v>
-      </c>
-      <c r="F2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Mở trình duyệt_x000d_
-Truy cập trang "http://thuvienso.actvn.edu.vn"_x000d_
-Chọn thẻ có id là "txtLoginUsername"_x000d_
-Gõ "CT020126"_x000d_
-Chọn thẻ có id là "txtLoginPassword"_x000d_
-Gõ "CT020126"_x000d_
-Bấm vào "Đăng nhập"</v>
+        <v>Không</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Truy cập trang https://actvn.edu.vn</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
       </c>
       <c r="G2" t="str">
-        <v>đăng nhập thành công</v>
+        <v>Trang hiển thị không lỗi, có tiêu đề, menu, banner, thông tin trang chủ</v>
       </c>
       <c r="H2" t="str">
-        <v>Kiểm tra thấy "Thiết lập tài khoản"</v>
+        <v>Kiểm tra thấy "tiêu đề"; Kiểm tra thấy "menu"; Kiểm tra thấy "banner"; Kiểm tra thấy "thông tin trang chủ"</v>
       </c>
       <c r="I2" t="str">
-        <v>Kiểm tra thấy "Thiết lập tài khoản"</v>
+        <v>Không thể thực hiện hành động "Kiểm tra thấy "tiêu đề""</v>
       </c>
       <c r="J2" t="str">
         <v/>
       </c>
       <c r="K2" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v/>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
-      <c r="R2" t="str">
-        <v/>
-      </c>
-      <c r="S2" t="str">
-        <v/>
-      </c>
-      <c r="T2" t="str">
-        <v/>
-      </c>
-      <c r="U2" t="str">
-        <v/>
-      </c>
-      <c r="V2" t="str">
-        <v/>
-      </c>
-      <c r="W2" t="str">
-        <v/>
-      </c>
-      <c r="X2" t="str">
-        <v/>
-      </c>
-      <c r="Y2" t="str">
-        <v/>
-      </c>
-      <c r="Z2" t="str">
-        <v/>
-      </c>
-      <c r="AA2" t="str">
-        <v/>
-      </c>
-      <c r="AB2" t="str">
-        <v/>
+        <v>FAIL</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -594,34 +483,25 @@
         <v>Click menu/mục tương ứng</v>
       </c>
       <c r="E3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Mở trình duyệt_x000d_
-2. Truy cập trang https://actvn.edu.vn_x000d_
-3. Hover vào mục 'Giới thiệu' trên navbar_x000d_
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Giới thiệu' trên navbar
 4. Click vào mục 'Liên hệ'</v>
       </c>
       <c r="F3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Mở trình duyệt_x000d_
-Truy cập trang "http://thuvienso.actvn.edu.vn"_x000d_
-Bấm vào "Thiết lập tài khoản"_x000d_
-Tải tệp "test.jpg" lên tại ô có id "txtFile"_x000d_
-Chọn thẻ có id là "txtLastname"_x000d_
-Gõ "Trần Văn"_x000d_
-Chọn thẻ có id là "txtFirstname"_x000d_
-Gõ "Huy"_x000d_
-Chọn "10" từ "ngày" được xổ xuống_x000d_
-Chọn "5" từ "tháng" được xổ xuống_x000d_
-Chọn "2003" từ "năm" được xổ xuống_x000d_
-Chọn radio "Nữ"_x000d_
-Bấm vào "Cập nhật"</v>
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Giới thiệu"
+Bấm vào "Liên hệ"</v>
       </c>
       <c r="G3" t="str">
-        <v>cập nhật thành công</v>
+        <v>Hiển thị địa chỉ, email, số điện thoại</v>
       </c>
       <c r="H3" t="str">
-        <v>Xuất hiện alert với nội dung là "Bạn cập nhật thành công", sau đó nhấn OK</v>
+        <v xml:space="preserve">        Kiểm tra thấy "Địa chỉ"; Kiểm tra thấy "Email"; Kiểm tra thấy "Điện thoại"</v>
       </c>
       <c r="I3" t="str">
-        <v>Xuất hiện alert với nội dung là "Bạn cập nhật thành công", sau đó nhấn OK</v>
+        <v xml:space="preserve">        Kiểm tra thấy "Địa chỉ"; Kiểm tra thấy "Email"; Kiểm tra thấy "Điện thoại"</v>
       </c>
       <c r="J3" t="str">
         <v/>
@@ -629,61 +509,930 @@
       <c r="K3" t="str">
         <v>PASS</v>
       </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
-        <v/>
-      </c>
-      <c r="N3" t="str">
-        <v/>
-      </c>
-      <c r="O3" t="str">
-        <v/>
-      </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
-      <c r="Q3" t="str">
-        <v/>
-      </c>
-      <c r="R3" t="str">
-        <v/>
-      </c>
-      <c r="S3" t="str">
-        <v/>
-      </c>
-      <c r="T3" t="str">
-        <v/>
-      </c>
-      <c r="U3" t="str">
-        <v/>
-      </c>
-      <c r="V3" t="str">
-        <v/>
-      </c>
-      <c r="W3" t="str">
-        <v/>
-      </c>
-      <c r="X3" t="str">
-        <v/>
-      </c>
-      <c r="Y3" t="str">
-        <v/>
-      </c>
-      <c r="Z3" t="str">
-        <v/>
-      </c>
-      <c r="AA3" t="str">
-        <v/>
-      </c>
-      <c r="AB3" t="str">
-        <v/>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>TC03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Kiểm tra điều hướng 'Mô hình đào tạo'</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Xác minh mục 'Mô hình đào tạo' hiển thị đúng</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Đào tạo' trên navbar
+4. Click vào 'Mô hình đào tạo'</v>
+      </c>
+      <c r="F4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Đào tạo"
+Bấm vào "Mô hình đào tạo"</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Trang mô tả mô hình hiển thị</v>
+      </c>
+      <c r="H4" t="str">
+        <v xml:space="preserve">        Kiểm tra thấy "Mô hình đào tạo"</v>
+      </c>
+      <c r="I4" t="str">
+        <v xml:space="preserve">        Kiểm tra thấy "Mô hình đào tạo"</v>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>TC04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Kiểm tra hiển thị file PDF của chương trình đào tạo ngành Công nghệ thông tin</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Đảm bảo khi nhấn vào liên kết, file PDF mở trực tiếp trên trình duyệt</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Đào tạo' trên navbar
+4. Click vào 'Chương trình đào tạo'
+5. Click vào 'Đại học Công nghệ thông tin'</v>
+      </c>
+      <c r="F5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Đào tạo"
+Bấm vào "Chương trình đào tạo"
+Bấm vào "Đại học Công nghệ thông tin"</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Trình duyệt mở tab mới hoặc chuyển trang hiển thị một file PDF, có nội dung chương trình đào tạo ngành CNTT</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Kiểm tra URL chứa "https://actvneduvn-my.sharepoint.com/personal/vinhlk_actvn_edu_vn/_layouts/15/onedrive.aspx?id=%2Fpersonal%2Fvinhlk%5Factvn%5Fedu%5Fvn%2FDocuments%2FC%C3%B4ng%20vi%E1%BB%87c%2FTin%20t%E1%BB%A9c%20Website%2FChuong%20trinh%20dao%20tao%20dai%20hoc%2FCh%C6%B0%C6%A1ng%20tr%C3%ACnh%20%C4%91%C3%A0o%20t%E1%BA%A1o%20ng%C3%A0nh%20C%C3%B4ng%20ngh%E1%BB%87%20th%C3%B4ng%20tin%2Epdf&amp;parent=%2Fpersonal%2Fvinhlk%5Factvn%5Fedu%5Fvn%2FDocuments%2FC%C3%B4ng%20vi%E1%BB%87c%2FTin%20t%E1%BB%A9c%20Website%2FChuong%20trinh%20dao%20tao%20dai%20hoc&amp;ga=1"</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Kiểm tra URL chứa "https://actvneduvn-my.sharepoint.com/personal/vinhlk_actvn_edu_vn/_layouts/15/onedrive.aspx?id=%2Fpersonal%2Fvinhlk%5Factvn%5Fedu%5Fvn%2FDocuments%2FC%C3%B4ng%20vi%E1%BB%87c%2FTin%20t%E1%BB%A9c%20Website%2FChuong%20trinh%20dao%20tao%20dai%20hoc%2FCh%C6%B0%C6%A1ng%20tr%C3%ACnh%20%C4%91%C3%A0o%20t%E1%BA%A1o%20ng%C3%A0nh%20C%C3%B4ng%20ngh%E1%BB%87%20th%C3%B4ng%20tin%2Epdf&amp;parent=%2Fpersonal%2Fvinhlk%5Factvn%5Fedu%5Fvn%2FDocuments%2FC%C3%B4ng%20vi%E1%BB%87c%2FTin%20t%E1%BB%A9c%20Website%2FChuong%20trinh%20dao%20tao%20dai%20hoc&amp;ga=1"</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>TC05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Kiểm tra 'Khảo thí &amp; ĐBCL'</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Đảm bảo có thông tin khảo thí</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Đào tạo' trên navbar
+4. Click vào 'Khảo thí và ĐBCL'</v>
+      </c>
+      <c r="F6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Đào tạo"
+Bấm vào "Khảo thí và ĐBCL"</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Thông tin khảo thí được hiển thị</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Kiểm tra URL chứa "ktdbcl.actvn.edu.vn"</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Kiểm tra URL chứa "ktdbcl.actvn.edu.vn"</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>TC06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Kiểm tra nội dung 'Tuyển sinh đại học'</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Xác minh nội dung tuyển sinh đại học hiển thị</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Tuyển sinh' trên navbar
+3. Click vào 'Tuyển sinh đại học'</v>
+      </c>
+      <c r="F7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Tuyển sinh"
+Bấm vào "Tuyển sinh đại học"</v>
+      </c>
+      <c r="G7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Trang đích có URL chứa “tuyensinh.actvn.edu.vn”, hiển thị tiêu đề hoặc nội dung liên quan đến tuyển sinh đại học như “Tuyển sinh” 
+</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Kiểm tra URL chứa "tuyensinh.actvn.edu.vn"; Kiểm tra thấy "Tuyển sinh"</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Kiểm tra URL chứa "tuyensinh.actvn.edu.vn"; Kiểm tra thấy "Tuyển sinh"</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>TC07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Kiểm tra 'Tuyển sinh sau đại học'</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Xác minh thông tin cao học có sẵn</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Tuyển sinh' trên navbar
+4. Click vào 'Tuyển sinh sau đại học'</v>
+      </c>
+      <c r="F8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Tuyển sinh"
+Bấm vào "Tuyển sinh sau đại học"</v>
+      </c>
+      <c r="G8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Trang đích có URL chứa “tuyensinh.actvn.edu.vn”, hiển thị tiêu đề hoặc nội dung liên quan đến tuyển sinh đại học như “Tuyển sinh” 
+</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Kiểm tra URL chứa "tuyensinh.actvn.edu.vn"; Kiểm tra thấy "Tuyển sinh"</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Kiểm tra URL chứa "tuyensinh.actvn.edu.vn"; Kiểm tra thấy "Tuyển sinh"</v>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>TC08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Kiểm tra truy cập 'Khoa ATTT'</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Đảm bảo truy cập khoa ATTT thành công</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Các khoa' trên navbar
+4. Click vào 'Khoa An toàn thông tin'</v>
+      </c>
+      <c r="F9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Các khoa"
+Bấm vào "Khoa An toàn thông tin"</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Hiển thị thông tin về khoa ATTT</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Kiểm tra thấy "khoa ATTT"</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Kiểm tra thấy "khoa ATTT"</v>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>TC09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Kiểm tra truy cập 'Khoa CNTT'</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Đảm bảo truy cập khoa CNTT thành công</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Các khoa' trên navbar
+4. Click vào 'Khoa Công nghệ thông tin'</v>
+      </c>
+      <c r="F10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Các khoa"
+Bấm vào "Khoa Công nghệ thông tin"</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Hiển thị thông tin về khoa CNTT</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Kiểm tra thấy "khoa CNTT"</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Không thể thực hiện hành động "Kiểm tra thấy "khoa CNTT""</v>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v>FAIL</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>TC10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Kiểm tra truy cập 'Khoa ĐTVT'</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Đảm bảo truy cập khoa ĐTVT thành công</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Các khoa' trên navbar
+4. Click vào 'Khoa Điện tử viễn thông'</v>
+      </c>
+      <c r="F11" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Các khoa"
+Bấm vào "Khoa Điện tử viễn thông"</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Hiển thị thông tin về khoa ĐTVT</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Kiểm tra URL chứa "https://dtvt.actvn.edu.vn/"</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Kiểm tra URL chứa "https://dtvt.actvn.edu.vn/"</v>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>TC11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Kiểm tra hiển thị 'Thông tin khoa học'</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Xác minh nội dung khoa học được hiển thị</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Nghiên cứu' trên navbar
+4. Click vào 'Thông tin khoa học'</v>
+      </c>
+      <c r="F12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Nghiên cứu"
+Bấm vào "Thông tin khoa học"</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Có thông tin nghiên cứu khoa học</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Kiểm tra thấy "Thông tin khoa học"</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Kiểm tra thấy "Thông tin khoa học"</v>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>TC12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Kiểm tra hiển thị thông tin 'Sinh viên NCKH'</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Đảm bảo có các bài viết dành cho sinh viên NCKH</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Nghiên cứu' trên navbar
+3. Click vào 'Sinh viên nghiên cứu khoa học'</v>
+      </c>
+      <c r="F13" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Nghiên cứu"
+Bấm vào "Sinh viên nghiên cứu khoa học"</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Hiển thị danh sách các bài viết liên quan đến NCKH dành cho sinh viên</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Kiểm tra thấy "Nghiên cứu khoa học dành  cho SV"</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Không thể thực hiện hành động "Kiểm tra thấy "Nghiên cứu khoa học dành  cho SV""</v>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v>FAIL</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>TC13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Kiểm tra hiển thị 'Thông báo sinh viên'</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Hiển thị các thông báo mới nhất cho SV</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Sinh viên' trên navbar
+4. Click vào 'Thông báo'</v>
+      </c>
+      <c r="F14" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Sinh viên"
+Bấm vào "Thông báo"</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Danh sách thông báo theo thời gian</v>
+      </c>
+      <c r="H14" t="str">
+        <v xml:space="preserve">        Kiểm tra thấy "THÔNG BÁO"</v>
+      </c>
+      <c r="I14" t="str">
+        <v xml:space="preserve">        Kiểm tra thấy "THÔNG BÁO"</v>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>TC14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Kiểm tra truy cập mục 'Học bổng'</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Xác minh nội dung học bổng hiện lên</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Sinh viên' trên navbar
+4. Click vào 'Học bổng'</v>
+      </c>
+      <c r="F15" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Sinh viên"
+Bấm vào "Học bổng"</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Hiển thị các học bổng hiện hành</v>
+      </c>
+      <c r="H15" t="str">
+        <v xml:space="preserve">        Kiểm tra thấy "Học bổng"</v>
+      </c>
+      <c r="I15" t="str">
+        <v xml:space="preserve">        Kiểm tra thấy "Học bổng"</v>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>TC15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Kiểm tra hiển thị văn bản - biểu mẫu</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Đảm bảo có thể tải văn bản, biểu mẫu</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Sinh viên' trên navbar
+4. Click vào 'Văn bản - Biểu mẫu'</v>
+      </c>
+      <c r="F16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Sinh viên"
+Bấm vào "Văn bản - Biểu mẫu"</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Hiển thị các file PDF, doc</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Kiểm tra URL chứa "https://actvneduvn-my.sharepoint.com/personal/support_actvn_edu_vn/_layouts/15/onedrive.aspx?id=%2Fpersonal%2Fsupport%5Factvn%5Fedu%5Fvn%2FDocuments%2FDocument&amp;ga=1"</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Kiểm tra URL chứa "https://actvneduvn-my.sharepoint.com/personal/support_actvn_edu_vn/_layouts/15/onedrive.aspx?id=%2Fpersonal%2Fsupport%5Factvn%5Fedu%5Fvn%2FDocuments%2FDocument&amp;ga=1"</v>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>TC16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Truy cập 'Thư viện số'</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Hiển thị tài liệu số cho sinh viên</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Thư viện' trên navbar
+4. Click vào 'Thư viện số'</v>
+      </c>
+      <c r="F17" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Thư viện"
+Bấm vào "Thư viện số"</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Điều hướng sang hệ thống thư viện</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Kiểm tra URL chứa "http://thuvienso.actvn.edu.vn/"</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Kiểm tra URL chứa "http://thuvienso.actvn.edu.vn/"</v>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>TC17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Truy cập 'Thư viện điện tử'</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Truy cập hệ thống thư viện số</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Thư viện' trên navbar
+4. Click vào 'Thư viện điện tử'</v>
+      </c>
+      <c r="F18" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Thư viện"
+Bấm vào "Thư viện điện tử"</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Điều hướng sang trang web của trung tâm thư viện https://thuvien.actvn.edu.vn/</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Kiểm tra URL chứa "https://thuvien.actvn.edu.vn/"</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Kiểm tra URL chứa "https://thuvien.actvn.edu.vn/"</v>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>TC18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Kiểm tra link đến 'Phân hiệu TP.HCM'</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Xác minh chuyển hướng đến trang phân hiệu</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Liên kết' trên navbar
+4. Click vào 'Phân hiệu tại TP.Hồ Chí Minh'</v>
+      </c>
+      <c r="F19" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Liên kết"
+Bấm vào "Phân hiệu tại TP.Hồ Chí Minh"</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Trang phân hiệu HCM được mở</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Kiểm tra URL chứa "https://hcmact.edu.vn/"</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Kiểm tra URL chứa "https://hcmact.edu.vn/"</v>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>TC19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Kiểm tra 'Đào tạo trực tuyến'</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Xác minh điều hướng đến hệ LMS</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Liên kết' trên navbar
+4. Click vào 'Đào tạo trực tuyến'</v>
+      </c>
+      <c r="F20" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Liên kết"
+Bấm vào "Đào tạo trực tuyến"</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Điều hướng đến nền tảng học trực tuyến https://portal.actvn.edu.vn/</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Kiểm tra URL chứa "https://portal.actvn.edu.vn/"</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Kiểm tra URL chứa "https://portal.actvn.edu.vn/"</v>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>TC20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Kiểm tra 'Tạp chí An toàn thông tin'</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Truy cập được tạp chí chuyên ngành</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Click menu/mục tương ứng</v>
+      </c>
+      <c r="E21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Mở trình duyệt
+2. Truy cập trang https://actvn.edu.vn
+3. Hover vào mục 'Liên kết' trên navbar
+4. Click vào 'Tạp chí An toàn thông tin'</v>
+      </c>
+      <c r="F21" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mở trình duyệt
+Truy cập trang https://actvn.edu.vn
+Di chuột đến "Liên kết"
+Bấm vào "Tạp chí An toàn thông tin"</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Điều hướng đến trang https://antoanthongtin.vn/</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Kiểm tra URL chứa "https://antoanthongtin.vn/"</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Kiểm tra URL chứa "https://antoanthongtin.vn/"</v>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>TC21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Kiểm tra chức năng tìm kiếm hợp lệ</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Đảm bảo hệ thống trả kết quả tìm kiếm đúng</v>
+      </c>
+      <c r="D22" t="str">
+        <v>"học bổng"</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Gõ “học bổng” → Enter</v>
+      </c>
+      <c r="F22" t="str" xml:space="preserve">
+        <v xml:space="preserve">Gõ "học bổng"
+Nhấn nút "Enter"</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Danh sách kết quả chứa từ “học bổng”</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Kiểm tra thấy "học bổng"</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Kiểm tra thấy "học bổng"</v>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>TC22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Tìm kiếm không hợp lệ</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Đảm bảo xử lý khi tìm từ không tồn tại</v>
+      </c>
+      <c r="D23" t="str">
+        <v>“abcdefxyz”</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Gõ “abcdefxyz” → Enter</v>
+      </c>
+      <c r="F23" t="str" xml:space="preserve">
+        <v xml:space="preserve">Gõ "abcdefxyz"
+Nhấn nút "Enter"</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Hiển thị “không có kết quả phù hợp” hoặc không hiển thị ra thông tin gì</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Kiểm tra thấy "không có kết quả phù hợp" hoặc không hiển thị gì</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Kiểm tra thấy "không có kết quả phù hợp" hoặc không hiển thị gì</v>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Kiểm tra hiển thị responsive</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Đảm bảo trang chủ hiển thị tốt trên mobile</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Không</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Mở trang ở kích thước 375x667</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Mở trang ở kích thước 375x667</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Menu chuyển thành biểu tượng ☰, nội dung gọn gàng</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Kiểm tra thấy "biểu tượng ☰" và nội dung gọn gàng</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Không thể thực hiện hành động "Kiểm tra thấy "biểu tượng ☰""</v>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v>FAIL</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Kiểm tra menu xổ xuống (dropdown)</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Kiểm tra các menu con hiển thị đúng</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Không</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Hover menu “Giới thiệu”</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Di chuột đến "Giới thiệu"</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Menu con hiển thị: “Logo học viện”, “Liên hệ”</v>
+      </c>
+      <c r="H25" t="str">
+        <v xml:space="preserve">        Kiểm tra thấy menu con "Logo học viện"; Kiểm tra thấy menu con "Liên hệ"</v>
+      </c>
+      <c r="I25" t="str">
+        <v xml:space="preserve">        Kiểm tra thấy menu con "Logo học viện"; Kiểm tra thấy menu con "Liên hệ"</v>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>TC25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Kiểm tra tốc độ tải trang</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Xác định trang chủ tải dưới 3s</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Không</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Truy cập trang chủ và đo thời gian load</v>
+      </c>
+      <c r="F26" t="str" xml:space="preserve">
+        <v xml:space="preserve">Truy cập trang chủ và đo thời gian load
+</v>
+      </c>
+      <c r="G26" t="str">
+        <v>window.performance.timing.loadEventEnd - navigationStart &lt; 3000 ms</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Kiểm tra thời gian tải trang &lt; 3000 ms</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Kiểm tra thời gian tải trang &lt; 3000 ms</v>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v>PASS</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>